<commit_message>
0326 - Cambios en login
</commit_message>
<xml_diff>
--- a/trabajadores/management/commands/nomina.xlsx
+++ b/trabajadores/management/commands/nomina.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dcarr\Desktop\ProG\genesis\trabajadores\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dcarr\Desktop\ProG\genesis\trabajadores\management\commands\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{08B0EF2A-92F8-4EE0-B8EA-FE9AE4BEAFCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C578010D-3EF7-4010-9549-2219610863D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{1C58C8FB-8A04-4B1C-A171-774073E551AA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="383">
   <si>
     <t xml:space="preserve">Nomina Personal Genesis </t>
   </si>
@@ -1181,6 +1181,15 @@
   </si>
   <si>
     <t>PRACTICANTE ELECTRICO</t>
+  </si>
+  <si>
+    <t>PRUEBA UNO SUJETO DE</t>
+  </si>
+  <si>
+    <t>12345678-9</t>
+  </si>
+  <si>
+    <t>TESTER</t>
   </si>
 </sst>
 </file>
@@ -1379,7 +1388,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1474,10 +1483,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2096,7 +2101,7 @@
       <c r="A2" s="1"/>
       <c r="B2" s="35">
         <f ca="1">+TODAY()</f>
-        <v>46104</v>
+        <v>46106</v>
       </c>
       <c r="C2" s="36"/>
       <c r="D2" s="36"/>
@@ -5877,13 +5882,13 @@
       <c r="A36" s="21">
         <v>32</v>
       </c>
-      <c r="B36" s="39" t="s">
+      <c r="B36" s="22" t="s">
         <v>343</v>
       </c>
-      <c r="C36" s="40" t="s">
+      <c r="C36" s="23" t="s">
         <v>344</v>
       </c>
-      <c r="D36" s="39" t="s">
+      <c r="D36" s="22" t="s">
         <v>345</v>
       </c>
     </row>
@@ -5891,13 +5896,13 @@
       <c r="A37" s="21">
         <v>33</v>
       </c>
-      <c r="B37" s="39" t="s">
+      <c r="B37" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C37" s="40" t="s">
+      <c r="C37" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="D37" s="39" t="s">
+      <c r="D37" s="22" t="s">
         <v>331</v>
       </c>
     </row>
@@ -5905,13 +5910,13 @@
       <c r="A38" s="21">
         <v>34</v>
       </c>
-      <c r="B38" s="39" t="s">
+      <c r="B38" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="C38" s="40" t="s">
+      <c r="C38" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="D38" s="39" t="s">
+      <c r="D38" s="22" t="s">
         <v>332</v>
       </c>
     </row>
@@ -5919,13 +5924,13 @@
       <c r="A39" s="21">
         <v>35</v>
       </c>
-      <c r="B39" s="39" t="s">
+      <c r="B39" s="22" t="s">
         <v>280</v>
       </c>
-      <c r="C39" s="40" t="s">
+      <c r="C39" s="23" t="s">
         <v>281</v>
       </c>
-      <c r="D39" s="39" t="s">
+      <c r="D39" s="22" t="s">
         <v>333</v>
       </c>
     </row>
@@ -5933,13 +5938,13 @@
       <c r="A40" s="21">
         <v>36</v>
       </c>
-      <c r="B40" s="39" t="s">
+      <c r="B40" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="C40" s="40" t="s">
+      <c r="C40" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="D40" s="39" t="s">
+      <c r="D40" s="22" t="s">
         <v>7</v>
       </c>
     </row>
@@ -5947,13 +5952,13 @@
       <c r="A41" s="21">
         <v>37</v>
       </c>
-      <c r="B41" s="39" t="s">
+      <c r="B41" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="C41" s="40" t="s">
+      <c r="C41" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="D41" s="39" t="s">
+      <c r="D41" s="22" t="s">
         <v>7</v>
       </c>
     </row>
@@ -5961,13 +5966,13 @@
       <c r="A42" s="21">
         <v>38</v>
       </c>
-      <c r="B42" s="39" t="s">
+      <c r="B42" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="C42" s="40" t="s">
+      <c r="C42" s="23" t="s">
         <v>208</v>
       </c>
-      <c r="D42" s="39" t="s">
+      <c r="D42" s="22" t="s">
         <v>141</v>
       </c>
     </row>
@@ -5975,13 +5980,13 @@
       <c r="A43" s="21">
         <v>39</v>
       </c>
-      <c r="B43" s="39" t="s">
+      <c r="B43" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="C43" s="40" t="s">
+      <c r="C43" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="D43" s="39" t="s">
+      <c r="D43" s="22" t="s">
         <v>141</v>
       </c>
     </row>
@@ -5989,13 +5994,13 @@
       <c r="A44" s="21">
         <v>40</v>
       </c>
-      <c r="B44" s="39" t="s">
+      <c r="B44" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="C44" s="40" t="s">
+      <c r="C44" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="D44" s="39" t="s">
+      <c r="D44" s="22" t="s">
         <v>90</v>
       </c>
     </row>
@@ -6003,13 +6008,13 @@
       <c r="A45" s="21">
         <v>41</v>
       </c>
-      <c r="B45" s="39" t="s">
+      <c r="B45" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="C45" s="40" t="s">
+      <c r="C45" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="D45" s="39" t="s">
+      <c r="D45" s="22" t="s">
         <v>96</v>
       </c>
     </row>
@@ -6017,13 +6022,13 @@
       <c r="A46" s="21">
         <v>42</v>
       </c>
-      <c r="B46" s="39" t="s">
+      <c r="B46" s="22" t="s">
         <v>348</v>
       </c>
-      <c r="C46" s="40" t="s">
+      <c r="C46" s="23" t="s">
         <v>349</v>
       </c>
-      <c r="D46" s="39" t="s">
+      <c r="D46" s="22" t="s">
         <v>350</v>
       </c>
     </row>
@@ -6031,13 +6036,13 @@
       <c r="A47" s="21">
         <v>43</v>
       </c>
-      <c r="B47" s="39" t="s">
+      <c r="B47" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="C47" s="40" t="s">
+      <c r="C47" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="D47" s="39" t="s">
+      <c r="D47" s="22" t="s">
         <v>103</v>
       </c>
     </row>
@@ -6045,13 +6050,13 @@
       <c r="A48" s="21">
         <v>44</v>
       </c>
-      <c r="B48" s="39" t="s">
+      <c r="B48" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="C48" s="40" t="s">
+      <c r="C48" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="D48" s="39" t="s">
+      <c r="D48" s="22" t="s">
         <v>334</v>
       </c>
     </row>
@@ -6059,13 +6064,13 @@
       <c r="A49" s="21">
         <v>45</v>
       </c>
-      <c r="B49" s="39" t="s">
+      <c r="B49" s="22" t="s">
         <v>355</v>
       </c>
-      <c r="C49" s="40" t="s">
+      <c r="C49" s="23" t="s">
         <v>356</v>
       </c>
-      <c r="D49" s="39" t="s">
+      <c r="D49" s="22" t="s">
         <v>103</v>
       </c>
     </row>
@@ -6073,13 +6078,13 @@
       <c r="A50" s="21">
         <v>46</v>
       </c>
-      <c r="B50" s="39" t="s">
+      <c r="B50" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="C50" s="40" t="s">
+      <c r="C50" s="23" t="s">
         <v>190</v>
       </c>
-      <c r="D50" s="39" t="s">
+      <c r="D50" s="22" t="s">
         <v>108</v>
       </c>
     </row>
@@ -6087,13 +6092,13 @@
       <c r="A51" s="21">
         <v>47</v>
       </c>
-      <c r="B51" s="39" t="s">
+      <c r="B51" s="22" t="s">
         <v>370</v>
       </c>
-      <c r="C51" s="40" t="s">
+      <c r="C51" s="23" t="s">
         <v>371</v>
       </c>
-      <c r="D51" s="39" t="s">
+      <c r="D51" s="22" t="s">
         <v>372</v>
       </c>
     </row>
@@ -6101,13 +6106,13 @@
       <c r="A52" s="21">
         <v>48</v>
       </c>
-      <c r="B52" s="39" t="s">
+      <c r="B52" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="C52" s="40" t="s">
+      <c r="C52" s="23" t="s">
         <v>251</v>
       </c>
-      <c r="D52" s="39" t="s">
+      <c r="D52" s="22" t="s">
         <v>293</v>
       </c>
     </row>
@@ -6115,13 +6120,13 @@
       <c r="A53" s="21">
         <v>49</v>
       </c>
-      <c r="B53" s="39" t="s">
+      <c r="B53" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="C53" s="40" t="s">
+      <c r="C53" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="D53" s="39" t="s">
+      <c r="D53" s="22" t="s">
         <v>68</v>
       </c>
     </row>
@@ -6129,13 +6134,13 @@
       <c r="A54" s="21">
         <v>50</v>
       </c>
-      <c r="B54" s="39" t="s">
+      <c r="B54" s="22" t="s">
         <v>324</v>
       </c>
-      <c r="C54" s="40" t="s">
+      <c r="C54" s="23" t="s">
         <v>325</v>
       </c>
-      <c r="D54" s="39" t="s">
+      <c r="D54" s="22" t="s">
         <v>141</v>
       </c>
     </row>
@@ -6143,13 +6148,13 @@
       <c r="A55" s="21">
         <v>51</v>
       </c>
-      <c r="B55" s="39" t="s">
+      <c r="B55" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="C55" s="40" t="s">
+      <c r="C55" s="23" t="s">
         <v>200</v>
       </c>
-      <c r="D55" s="39" t="s">
+      <c r="D55" s="22" t="s">
         <v>108</v>
       </c>
     </row>
@@ -6157,13 +6162,13 @@
       <c r="A56" s="21">
         <v>52</v>
       </c>
-      <c r="B56" s="39" t="s">
+      <c r="B56" s="22" t="s">
         <v>346</v>
       </c>
-      <c r="C56" s="40" t="s">
+      <c r="C56" s="23" t="s">
         <v>347</v>
       </c>
-      <c r="D56" s="39" t="s">
+      <c r="D56" s="22" t="s">
         <v>103</v>
       </c>
     </row>
@@ -6171,13 +6176,13 @@
       <c r="A57" s="21">
         <v>53</v>
       </c>
-      <c r="B57" s="39" t="s">
+      <c r="B57" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="C57" s="40" t="s">
+      <c r="C57" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="D57" s="39" t="s">
+      <c r="D57" s="22" t="s">
         <v>300</v>
       </c>
     </row>
@@ -6185,13 +6190,13 @@
       <c r="A58" s="21">
         <v>54</v>
       </c>
-      <c r="B58" s="39" t="s">
+      <c r="B58" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C58" s="40" t="s">
+      <c r="C58" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="D58" s="39" t="s">
+      <c r="D58" s="22" t="s">
         <v>113</v>
       </c>
     </row>
@@ -6199,13 +6204,13 @@
       <c r="A59" s="21">
         <v>55</v>
       </c>
-      <c r="B59" s="39" t="s">
+      <c r="B59" s="22" t="s">
         <v>254</v>
       </c>
-      <c r="C59" s="40" t="s">
+      <c r="C59" s="23" t="s">
         <v>255</v>
       </c>
-      <c r="D59" s="39" t="s">
+      <c r="D59" s="22" t="s">
         <v>90</v>
       </c>
     </row>
@@ -6213,13 +6218,13 @@
       <c r="A60" s="21">
         <v>56</v>
       </c>
-      <c r="B60" s="39" t="s">
+      <c r="B60" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="C60" s="40" t="s">
+      <c r="C60" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="D60" s="39" t="s">
+      <c r="D60" s="22" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6227,13 +6232,13 @@
       <c r="A61" s="21">
         <v>57</v>
       </c>
-      <c r="B61" s="39" t="s">
+      <c r="B61" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="C61" s="40" t="s">
+      <c r="C61" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="D61" s="39" t="s">
+      <c r="D61" s="22" t="s">
         <v>120</v>
       </c>
     </row>
@@ -6241,13 +6246,13 @@
       <c r="A62" s="21">
         <v>58</v>
       </c>
-      <c r="B62" s="39" t="s">
+      <c r="B62" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="C62" s="40" t="s">
+      <c r="C62" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="D62" s="39" t="s">
+      <c r="D62" s="22" t="s">
         <v>300</v>
       </c>
     </row>
@@ -6255,13 +6260,13 @@
       <c r="A63" s="21">
         <v>59</v>
       </c>
-      <c r="B63" s="39" t="s">
+      <c r="B63" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="C63" s="40" t="s">
+      <c r="C63" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="D63" s="39" t="s">
+      <c r="D63" s="22" t="s">
         <v>108</v>
       </c>
     </row>
@@ -6269,13 +6274,13 @@
       <c r="A64" s="21">
         <v>60</v>
       </c>
-      <c r="B64" s="39" t="s">
+      <c r="B64" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="C64" s="40" t="s">
+      <c r="C64" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="D64" s="39" t="s">
+      <c r="D64" s="22" t="s">
         <v>68</v>
       </c>
     </row>
@@ -6283,13 +6288,13 @@
       <c r="A65" s="21">
         <v>61</v>
       </c>
-      <c r="B65" s="39" t="s">
+      <c r="B65" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="C65" s="40" t="s">
+      <c r="C65" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="D65" s="39" t="s">
+      <c r="D65" s="22" t="s">
         <v>103</v>
       </c>
     </row>
@@ -6297,13 +6302,13 @@
       <c r="A66" s="21">
         <v>62</v>
       </c>
-      <c r="B66" s="39" t="s">
+      <c r="B66" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="C66" s="40" t="s">
+      <c r="C66" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="D66" s="39" t="s">
+      <c r="D66" s="22" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6311,13 +6316,13 @@
       <c r="A67" s="21">
         <v>63</v>
       </c>
-      <c r="B67" s="39" t="s">
+      <c r="B67" s="22" t="s">
         <v>351</v>
       </c>
-      <c r="C67" s="40" t="s">
+      <c r="C67" s="23" t="s">
         <v>352</v>
       </c>
-      <c r="D67" s="39" t="s">
+      <c r="D67" s="22" t="s">
         <v>350</v>
       </c>
     </row>
@@ -6325,13 +6330,13 @@
       <c r="A68" s="21">
         <v>64</v>
       </c>
-      <c r="B68" s="39" t="s">
+      <c r="B68" s="22" t="s">
         <v>365</v>
       </c>
-      <c r="C68" s="40" t="s">
+      <c r="C68" s="23" t="s">
         <v>366</v>
       </c>
-      <c r="D68" s="39" t="s">
+      <c r="D68" s="22" t="s">
         <v>367</v>
       </c>
     </row>
@@ -6339,13 +6344,13 @@
       <c r="A69" s="21">
         <v>65</v>
       </c>
-      <c r="B69" s="39" t="s">
+      <c r="B69" s="22" t="s">
         <v>357</v>
       </c>
-      <c r="C69" s="40" t="s">
+      <c r="C69" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="D69" s="39" t="s">
+      <c r="D69" s="22" t="s">
         <v>227</v>
       </c>
     </row>
@@ -6353,13 +6358,13 @@
       <c r="A70" s="21">
         <v>66</v>
       </c>
-      <c r="B70" s="39" t="s">
+      <c r="B70" s="22" t="s">
         <v>368</v>
       </c>
-      <c r="C70" s="40" t="s">
+      <c r="C70" s="23" t="s">
         <v>369</v>
       </c>
-      <c r="D70" s="39" t="s">
+      <c r="D70" s="22" t="s">
         <v>367</v>
       </c>
     </row>
@@ -6367,13 +6372,13 @@
       <c r="A71" s="21">
         <v>67</v>
       </c>
-      <c r="B71" s="39" t="s">
+      <c r="B71" s="22" t="s">
         <v>338</v>
       </c>
-      <c r="C71" s="40" t="s">
+      <c r="C71" s="23" t="s">
         <v>339</v>
       </c>
-      <c r="D71" s="39" t="s">
+      <c r="D71" s="22" t="s">
         <v>340</v>
       </c>
     </row>
@@ -6381,13 +6386,13 @@
       <c r="A72" s="21">
         <v>68</v>
       </c>
-      <c r="B72" s="39" t="s">
+      <c r="B72" s="22" t="s">
         <v>260</v>
       </c>
-      <c r="C72" s="40" t="s">
+      <c r="C72" s="23" t="s">
         <v>261</v>
       </c>
-      <c r="D72" s="39" t="s">
+      <c r="D72" s="22" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6395,13 +6400,13 @@
       <c r="A73" s="21">
         <v>69</v>
       </c>
-      <c r="B73" s="39" t="s">
+      <c r="B73" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="C73" s="40" t="s">
+      <c r="C73" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="D73" s="39" t="s">
+      <c r="D73" s="22" t="s">
         <v>141</v>
       </c>
     </row>
@@ -6409,13 +6414,13 @@
       <c r="A74" s="21">
         <v>70</v>
       </c>
-      <c r="B74" s="39" t="s">
+      <c r="B74" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="C74" s="40" t="s">
+      <c r="C74" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="D74" s="39" t="s">
+      <c r="D74" s="22" t="s">
         <v>141</v>
       </c>
     </row>
@@ -6423,13 +6428,13 @@
       <c r="A75" s="21">
         <v>71</v>
       </c>
-      <c r="B75" s="39" t="s">
+      <c r="B75" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="C75" s="40" t="s">
+      <c r="C75" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="D75" s="39" t="s">
+      <c r="D75" s="22" t="s">
         <v>335</v>
       </c>
     </row>
@@ -6437,13 +6442,13 @@
       <c r="A76" s="21">
         <v>72</v>
       </c>
-      <c r="B76" s="39" t="s">
+      <c r="B76" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="C76" s="40" t="s">
+      <c r="C76" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="D76" s="39" t="s">
+      <c r="D76" s="22" t="s">
         <v>336</v>
       </c>
     </row>
@@ -6451,13 +6456,13 @@
       <c r="A77" s="21">
         <v>73</v>
       </c>
-      <c r="B77" s="39" t="s">
+      <c r="B77" s="22" t="s">
         <v>272</v>
       </c>
-      <c r="C77" s="40" t="s">
+      <c r="C77" s="23" t="s">
         <v>273</v>
       </c>
-      <c r="D77" s="39" t="s">
+      <c r="D77" s="22" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6465,13 +6470,13 @@
       <c r="A78" s="21">
         <v>74</v>
       </c>
-      <c r="B78" s="39" t="s">
+      <c r="B78" s="22" t="s">
         <v>294</v>
       </c>
-      <c r="C78" s="40" t="s">
+      <c r="C78" s="23" t="s">
         <v>295</v>
       </c>
-      <c r="D78" s="39" t="s">
+      <c r="D78" s="22" t="s">
         <v>155</v>
       </c>
     </row>
@@ -6479,13 +6484,13 @@
       <c r="A79" s="21">
         <v>75</v>
       </c>
-      <c r="B79" s="39" t="s">
+      <c r="B79" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="C79" s="40" t="s">
+      <c r="C79" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="D79" s="39" t="s">
+      <c r="D79" s="22" t="s">
         <v>103</v>
       </c>
     </row>
@@ -6493,13 +6498,13 @@
       <c r="A80" s="21">
         <v>76</v>
       </c>
-      <c r="B80" s="39" t="s">
+      <c r="B80" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="C80" s="40" t="s">
+      <c r="C80" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="D80" s="39" t="s">
+      <c r="D80" s="22" t="s">
         <v>103</v>
       </c>
     </row>
@@ -6507,13 +6512,13 @@
       <c r="A81" s="21">
         <v>77</v>
       </c>
-      <c r="B81" s="39" t="s">
+      <c r="B81" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="C81" s="40" t="s">
+      <c r="C81" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="D81" s="39" t="s">
+      <c r="D81" s="22" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6521,13 +6526,13 @@
       <c r="A82" s="21">
         <v>78</v>
       </c>
-      <c r="B82" s="39" t="s">
+      <c r="B82" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="C82" s="40" t="s">
+      <c r="C82" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="D82" s="39" t="s">
+      <c r="D82" s="22" t="s">
         <v>103</v>
       </c>
     </row>
@@ -6535,13 +6540,13 @@
       <c r="A83" s="21">
         <v>79</v>
       </c>
-      <c r="B83" s="39" t="s">
+      <c r="B83" s="22" t="s">
         <v>363</v>
       </c>
-      <c r="C83" s="40" t="s">
+      <c r="C83" s="23" t="s">
         <v>364</v>
       </c>
-      <c r="D83" s="39" t="s">
+      <c r="D83" s="22" t="s">
         <v>90</v>
       </c>
     </row>
@@ -6549,13 +6554,13 @@
       <c r="A84" s="21">
         <v>80</v>
       </c>
-      <c r="B84" s="39" t="s">
+      <c r="B84" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="C84" s="40" t="s">
+      <c r="C84" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="D84" s="39" t="s">
+      <c r="D84" s="22" t="s">
         <v>166</v>
       </c>
     </row>
@@ -6563,13 +6568,13 @@
       <c r="A85" s="21">
         <v>81</v>
       </c>
-      <c r="B85" s="39" t="s">
+      <c r="B85" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="C85" s="40" t="s">
+      <c r="C85" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="D85" s="39" t="s">
+      <c r="D85" s="22" t="s">
         <v>332</v>
       </c>
     </row>
@@ -6577,13 +6582,13 @@
       <c r="A86" s="21">
         <v>82</v>
       </c>
-      <c r="B86" s="39" t="s">
+      <c r="B86" s="22" t="s">
         <v>171</v>
       </c>
-      <c r="C86" s="40" t="s">
+      <c r="C86" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="D86" s="39" t="s">
+      <c r="D86" s="22" t="s">
         <v>49</v>
       </c>
     </row>
@@ -6591,13 +6596,13 @@
       <c r="A87" s="21">
         <v>83</v>
       </c>
-      <c r="B87" s="39" t="s">
+      <c r="B87" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="C87" s="40" t="s">
+      <c r="C87" s="23" t="s">
         <v>174</v>
       </c>
-      <c r="D87" s="39" t="s">
+      <c r="D87" s="22" t="s">
         <v>332</v>
       </c>
     </row>
@@ -6605,13 +6610,13 @@
       <c r="A88" s="21">
         <v>84</v>
       </c>
-      <c r="B88" s="39" t="s">
+      <c r="B88" s="22" t="s">
         <v>175</v>
       </c>
-      <c r="C88" s="40" t="s">
+      <c r="C88" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="D88" s="39" t="s">
+      <c r="D88" s="22" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6619,13 +6624,13 @@
       <c r="A89" s="21">
         <v>85</v>
       </c>
-      <c r="B89" s="39" t="s">
+      <c r="B89" s="22" t="s">
         <v>177</v>
       </c>
-      <c r="C89" s="40" t="s">
+      <c r="C89" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="D89" s="39" t="s">
+      <c r="D89" s="22" t="s">
         <v>227</v>
       </c>
     </row>
@@ -6633,21 +6638,29 @@
       <c r="A90" s="21">
         <v>86</v>
       </c>
-      <c r="B90" s="39" t="s">
+      <c r="B90" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="C90" s="40" t="s">
+      <c r="C90" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="D90" s="39" t="s">
+      <c r="D90" s="22" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="21"/>
-      <c r="B91" s="39"/>
-      <c r="C91" s="40"/>
-      <c r="D91" s="39"/>
+      <c r="A91" s="21">
+        <v>87</v>
+      </c>
+      <c r="B91" s="22" t="s">
+        <v>380</v>
+      </c>
+      <c r="C91" s="23" t="s">
+        <v>381</v>
+      </c>
+      <c r="D91" s="22" t="s">
+        <v>382</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>